<commit_message>
message validation en francais
</commit_message>
<xml_diff>
--- a/public/docs/import_prospects.xlsx
+++ b/public/docs/import_prospects.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\FADWA\ERP\api_0.1\public\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{032230F2-A0CC-4A59-A006-45FEC1DA6BA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C95341B9-CEC3-4781-890F-F2BE9A2F4B22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{9D75755E-FE6E-4BAB-BDD4-4CD9ECED924A}"/>
+    <workbookView xWindow="50" yWindow="1900" windowWidth="19150" windowHeight="7360" xr2:uid="{9D75755E-FE6E-4BAB-BDD4-4CD9ECED924A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>cin</t>
   </si>
@@ -73,6 +73,9 @@
   </si>
   <si>
     <t>+212678655997</t>
+  </si>
+  <si>
+    <t>partenaire</t>
   </si>
 </sst>
 </file>
@@ -443,14 +446,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E0F0443-92CC-4029-AE8D-C9742B61B601}">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="4" max="4" width="34.453125" customWidth="1"/>
     <col min="5" max="5" width="23.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -475,8 +478,11 @@
       <c r="H1" s="1" t="s">
         <v>12</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>7</v>
       </c>

</xml_diff>